<commit_message>
added new code to check data and fix error with 2009
</commit_message>
<xml_diff>
--- a/Excel Files IPEDS/Trimmed_OLD/c2000_trimmed_file.xlsx
+++ b/Excel Files IPEDS/Trimmed_OLD/c2000_trimmed_file.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E376"/>
+  <dimension ref="A1:G376"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,6 +451,16 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>crace15</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>crace16</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Year</t>
         </is>
       </c>
@@ -469,6 +479,12 @@
         <v>7</v>
       </c>
       <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -486,6 +502,12 @@
         <v>7</v>
       </c>
       <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -503,6 +525,12 @@
         <v>9</v>
       </c>
       <c r="E4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -520,6 +548,12 @@
         <v>7</v>
       </c>
       <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -537,6 +571,12 @@
         <v>9</v>
       </c>
       <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -554,6 +594,12 @@
         <v>7</v>
       </c>
       <c r="E7" t="n">
+        <v>7</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -571,6 +617,12 @@
         <v>9</v>
       </c>
       <c r="E8" t="n">
+        <v>11</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -588,6 +640,12 @@
         <v>9</v>
       </c>
       <c r="E9" t="n">
+        <v>8</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -605,6 +663,12 @@
         <v>9</v>
       </c>
       <c r="E10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -622,6 +686,12 @@
         <v>7</v>
       </c>
       <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -639,6 +709,12 @@
         <v>7</v>
       </c>
       <c r="E12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -656,6 +732,12 @@
         <v>7</v>
       </c>
       <c r="E13" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -673,6 +755,12 @@
         <v>9</v>
       </c>
       <c r="E14" t="n">
+        <v>5</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -690,6 +778,12 @@
         <v>7</v>
       </c>
       <c r="E15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F15" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -707,6 +801,12 @@
         <v>7</v>
       </c>
       <c r="E16" t="n">
+        <v>6</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -724,6 +824,12 @@
         <v>9</v>
       </c>
       <c r="E17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -741,6 +847,12 @@
         <v>7</v>
       </c>
       <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -758,6 +870,12 @@
         <v>9</v>
       </c>
       <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -775,6 +893,12 @@
         <v>7</v>
       </c>
       <c r="E20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -792,6 +916,12 @@
         <v>7</v>
       </c>
       <c r="E21" t="n">
+        <v>10</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -809,6 +939,12 @@
         <v>9</v>
       </c>
       <c r="E22" t="n">
+        <v>9</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -826,6 +962,12 @@
         <v>7</v>
       </c>
       <c r="E23" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -843,6 +985,12 @@
         <v>9</v>
       </c>
       <c r="E24" t="n">
+        <v>6</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -860,6 +1008,12 @@
         <v>9</v>
       </c>
       <c r="E25" t="n">
+        <v>6</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -877,6 +1031,12 @@
         <v>7</v>
       </c>
       <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -894,6 +1054,12 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
+        <v>7</v>
+      </c>
+      <c r="F27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -911,6 +1077,12 @@
         <v>9</v>
       </c>
       <c r="E28" t="n">
+        <v>4</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -928,6 +1100,12 @@
         <v>7</v>
       </c>
       <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -945,6 +1123,12 @@
         <v>7</v>
       </c>
       <c r="E30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -962,6 +1146,12 @@
         <v>7</v>
       </c>
       <c r="E31" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" t="n">
+        <v>2</v>
+      </c>
+      <c r="G31" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -979,6 +1169,12 @@
         <v>9</v>
       </c>
       <c r="E32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -996,6 +1192,12 @@
         <v>7</v>
       </c>
       <c r="E33" t="n">
+        <v>5</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1013,6 +1215,12 @@
         <v>9</v>
       </c>
       <c r="E34" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1030,6 +1238,12 @@
         <v>7</v>
       </c>
       <c r="E35" t="n">
+        <v>12</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1047,6 +1261,12 @@
         <v>9</v>
       </c>
       <c r="E36" t="n">
+        <v>14</v>
+      </c>
+      <c r="F36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1064,6 +1284,12 @@
         <v>7</v>
       </c>
       <c r="E37" t="n">
+        <v>4</v>
+      </c>
+      <c r="F37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G37" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1081,6 +1307,12 @@
         <v>7</v>
       </c>
       <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1098,6 +1330,12 @@
         <v>7</v>
       </c>
       <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1115,6 +1353,12 @@
         <v>9</v>
       </c>
       <c r="E40" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1132,6 +1376,12 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1149,6 +1399,12 @@
         <v>7</v>
       </c>
       <c r="E42" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1166,6 +1422,12 @@
         <v>9</v>
       </c>
       <c r="E43" t="n">
+        <v>4</v>
+      </c>
+      <c r="F43" t="n">
+        <v>2</v>
+      </c>
+      <c r="G43" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1183,6 +1445,12 @@
         <v>9</v>
       </c>
       <c r="E44" t="n">
+        <v>5</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1200,6 +1468,12 @@
         <v>7</v>
       </c>
       <c r="E45" t="n">
+        <v>4</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1217,6 +1491,12 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
+        <v>4</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1234,6 +1514,12 @@
         <v>7</v>
       </c>
       <c r="E47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1251,6 +1537,12 @@
         <v>9</v>
       </c>
       <c r="E48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1268,6 +1560,12 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1285,6 +1583,12 @@
         <v>9</v>
       </c>
       <c r="E50" t="n">
+        <v>2</v>
+      </c>
+      <c r="F50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1302,6 +1606,12 @@
         <v>9</v>
       </c>
       <c r="E51" t="n">
+        <v>4</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1319,6 +1629,12 @@
         <v>7</v>
       </c>
       <c r="E52" t="n">
+        <v>4</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1336,6 +1652,12 @@
         <v>9</v>
       </c>
       <c r="E53" t="n">
+        <v>8</v>
+      </c>
+      <c r="F53" t="n">
+        <v>2</v>
+      </c>
+      <c r="G53" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1353,6 +1675,12 @@
         <v>7</v>
       </c>
       <c r="E54" t="n">
+        <v>7</v>
+      </c>
+      <c r="F54" t="n">
+        <v>3</v>
+      </c>
+      <c r="G54" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1370,6 +1698,12 @@
         <v>9</v>
       </c>
       <c r="E55" t="n">
+        <v>6</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1387,6 +1721,12 @@
         <v>7</v>
       </c>
       <c r="E56" t="n">
+        <v>5</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1404,6 +1744,12 @@
         <v>7</v>
       </c>
       <c r="E57" t="n">
+        <v>2</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1421,6 +1767,12 @@
         <v>7</v>
       </c>
       <c r="E58" t="n">
+        <v>5</v>
+      </c>
+      <c r="F58" t="n">
+        <v>3</v>
+      </c>
+      <c r="G58" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1438,6 +1790,12 @@
         <v>7</v>
       </c>
       <c r="E59" t="n">
+        <v>6</v>
+      </c>
+      <c r="F59" t="n">
+        <v>2</v>
+      </c>
+      <c r="G59" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1455,6 +1813,12 @@
         <v>9</v>
       </c>
       <c r="E60" t="n">
+        <v>6</v>
+      </c>
+      <c r="F60" t="n">
+        <v>2</v>
+      </c>
+      <c r="G60" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1472,6 +1836,12 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
+        <v>3</v>
+      </c>
+      <c r="F61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1489,6 +1859,12 @@
         <v>9</v>
       </c>
       <c r="E62" t="n">
+        <v>4</v>
+      </c>
+      <c r="F62" t="n">
+        <v>2</v>
+      </c>
+      <c r="G62" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1506,6 +1882,12 @@
         <v>7</v>
       </c>
       <c r="E63" t="n">
+        <v>3</v>
+      </c>
+      <c r="F63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G63" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1523,6 +1905,12 @@
         <v>7</v>
       </c>
       <c r="E64" t="n">
+        <v>2</v>
+      </c>
+      <c r="F64" t="n">
+        <v>2</v>
+      </c>
+      <c r="G64" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1540,6 +1928,12 @@
         <v>9</v>
       </c>
       <c r="E65" t="n">
+        <v>6</v>
+      </c>
+      <c r="F65" t="n">
+        <v>2</v>
+      </c>
+      <c r="G65" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1557,6 +1951,12 @@
         <v>7</v>
       </c>
       <c r="E66" t="n">
+        <v>10</v>
+      </c>
+      <c r="F66" t="n">
+        <v>7</v>
+      </c>
+      <c r="G66" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1574,6 +1974,12 @@
         <v>9</v>
       </c>
       <c r="E67" t="n">
+        <v>14</v>
+      </c>
+      <c r="F67" t="n">
+        <v>3</v>
+      </c>
+      <c r="G67" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1591,6 +1997,12 @@
         <v>7</v>
       </c>
       <c r="E68" t="n">
+        <v>12</v>
+      </c>
+      <c r="F68" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1608,6 +2020,12 @@
         <v>9</v>
       </c>
       <c r="E69" t="n">
+        <v>14</v>
+      </c>
+      <c r="F69" t="n">
+        <v>3</v>
+      </c>
+      <c r="G69" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1625,6 +2043,12 @@
         <v>7</v>
       </c>
       <c r="E70" t="n">
+        <v>2</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1642,6 +2066,12 @@
         <v>7</v>
       </c>
       <c r="E71" t="n">
+        <v>12</v>
+      </c>
+      <c r="F71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G71" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1659,6 +2089,12 @@
         <v>9</v>
       </c>
       <c r="E72" t="n">
+        <v>15</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1676,6 +2112,12 @@
         <v>9</v>
       </c>
       <c r="E73" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1693,6 +2135,12 @@
         <v>7</v>
       </c>
       <c r="E74" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1710,6 +2158,12 @@
         <v>7</v>
       </c>
       <c r="E75" t="n">
+        <v>3</v>
+      </c>
+      <c r="F75" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1727,6 +2181,12 @@
         <v>9</v>
       </c>
       <c r="E76" t="n">
+        <v>5</v>
+      </c>
+      <c r="F76" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1744,6 +2204,12 @@
         <v>9</v>
       </c>
       <c r="E77" t="n">
+        <v>4</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1761,6 +2227,12 @@
         <v>7</v>
       </c>
       <c r="E78" t="n">
+        <v>3</v>
+      </c>
+      <c r="F78" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1778,6 +2250,12 @@
         <v>7</v>
       </c>
       <c r="E79" t="n">
+        <v>1</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1795,6 +2273,12 @@
         <v>9</v>
       </c>
       <c r="E80" t="n">
+        <v>12</v>
+      </c>
+      <c r="F80" t="n">
+        <v>2</v>
+      </c>
+      <c r="G80" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1812,6 +2296,12 @@
         <v>7</v>
       </c>
       <c r="E81" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" t="n">
+        <v>1</v>
+      </c>
+      <c r="G81" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1829,6 +2319,12 @@
         <v>7</v>
       </c>
       <c r="E82" t="n">
+        <v>1</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1846,6 +2342,12 @@
         <v>7</v>
       </c>
       <c r="E83" t="n">
+        <v>15</v>
+      </c>
+      <c r="F83" t="n">
+        <v>1</v>
+      </c>
+      <c r="G83" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1863,6 +2365,12 @@
         <v>9</v>
       </c>
       <c r="E84" t="n">
+        <v>18</v>
+      </c>
+      <c r="F84" t="n">
+        <v>5</v>
+      </c>
+      <c r="G84" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1880,6 +2388,12 @@
         <v>7</v>
       </c>
       <c r="E85" t="n">
+        <v>11</v>
+      </c>
+      <c r="F85" t="n">
+        <v>2</v>
+      </c>
+      <c r="G85" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1897,6 +2411,12 @@
         <v>9</v>
       </c>
       <c r="E86" t="n">
+        <v>13</v>
+      </c>
+      <c r="F86" t="n">
+        <v>2</v>
+      </c>
+      <c r="G86" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1914,6 +2434,12 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
+        <v>1</v>
+      </c>
+      <c r="F87" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1931,6 +2457,12 @@
         <v>9</v>
       </c>
       <c r="E88" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1948,6 +2480,12 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
+        <v>1</v>
+      </c>
+      <c r="F89" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1965,6 +2503,12 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
+        <v>5</v>
+      </c>
+      <c r="F90" t="n">
+        <v>2</v>
+      </c>
+      <c r="G90" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1982,6 +2526,12 @@
         <v>9</v>
       </c>
       <c r="E91" t="n">
+        <v>3</v>
+      </c>
+      <c r="F91" t="n">
+        <v>1</v>
+      </c>
+      <c r="G91" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1999,6 +2549,12 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
+        <v>1</v>
+      </c>
+      <c r="F92" t="n">
+        <v>1</v>
+      </c>
+      <c r="G92" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2016,6 +2572,12 @@
         <v>9</v>
       </c>
       <c r="E93" t="n">
+        <v>4</v>
+      </c>
+      <c r="F93" t="n">
+        <v>1</v>
+      </c>
+      <c r="G93" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2033,6 +2595,12 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
+        <v>6</v>
+      </c>
+      <c r="F94" t="n">
+        <v>2</v>
+      </c>
+      <c r="G94" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2050,6 +2618,12 @@
         <v>9</v>
       </c>
       <c r="E95" t="n">
+        <v>1</v>
+      </c>
+      <c r="F95" t="n">
+        <v>1</v>
+      </c>
+      <c r="G95" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2067,6 +2641,12 @@
         <v>7</v>
       </c>
       <c r="E96" t="n">
+        <v>1</v>
+      </c>
+      <c r="F96" t="n">
+        <v>0</v>
+      </c>
+      <c r="G96" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2084,6 +2664,12 @@
         <v>9</v>
       </c>
       <c r="E97" t="n">
+        <v>3</v>
+      </c>
+      <c r="F97" t="n">
+        <v>0</v>
+      </c>
+      <c r="G97" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2101,6 +2687,12 @@
         <v>7</v>
       </c>
       <c r="E98" t="n">
+        <v>3</v>
+      </c>
+      <c r="F98" t="n">
+        <v>0</v>
+      </c>
+      <c r="G98" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2118,6 +2710,12 @@
         <v>9</v>
       </c>
       <c r="E99" t="n">
+        <v>10</v>
+      </c>
+      <c r="F99" t="n">
+        <v>1</v>
+      </c>
+      <c r="G99" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2135,6 +2733,12 @@
         <v>7</v>
       </c>
       <c r="E100" t="n">
+        <v>6</v>
+      </c>
+      <c r="F100" t="n">
+        <v>0</v>
+      </c>
+      <c r="G100" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2152,6 +2756,12 @@
         <v>9</v>
       </c>
       <c r="E101" t="n">
+        <v>9</v>
+      </c>
+      <c r="F101" t="n">
+        <v>4</v>
+      </c>
+      <c r="G101" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2169,6 +2779,12 @@
         <v>7</v>
       </c>
       <c r="E102" t="n">
+        <v>2</v>
+      </c>
+      <c r="F102" t="n">
+        <v>0</v>
+      </c>
+      <c r="G102" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2186,6 +2802,12 @@
         <v>9</v>
       </c>
       <c r="E103" t="n">
+        <v>2</v>
+      </c>
+      <c r="F103" t="n">
+        <v>0</v>
+      </c>
+      <c r="G103" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2203,6 +2825,12 @@
         <v>9</v>
       </c>
       <c r="E104" t="n">
+        <v>1</v>
+      </c>
+      <c r="F104" t="n">
+        <v>0</v>
+      </c>
+      <c r="G104" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2220,6 +2848,12 @@
         <v>7</v>
       </c>
       <c r="E105" t="n">
+        <v>1</v>
+      </c>
+      <c r="F105" t="n">
+        <v>0</v>
+      </c>
+      <c r="G105" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2237,6 +2871,12 @@
         <v>7</v>
       </c>
       <c r="E106" t="n">
+        <v>2</v>
+      </c>
+      <c r="F106" t="n">
+        <v>1</v>
+      </c>
+      <c r="G106" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2254,6 +2894,12 @@
         <v>9</v>
       </c>
       <c r="E107" t="n">
+        <v>3</v>
+      </c>
+      <c r="F107" t="n">
+        <v>0</v>
+      </c>
+      <c r="G107" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2271,6 +2917,12 @@
         <v>7</v>
       </c>
       <c r="E108" t="n">
+        <v>4</v>
+      </c>
+      <c r="F108" t="n">
+        <v>0</v>
+      </c>
+      <c r="G108" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2288,6 +2940,12 @@
         <v>7</v>
       </c>
       <c r="E109" t="n">
+        <v>0</v>
+      </c>
+      <c r="F109" t="n">
+        <v>1</v>
+      </c>
+      <c r="G109" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2305,6 +2963,12 @@
         <v>7</v>
       </c>
       <c r="E110" t="n">
+        <v>8</v>
+      </c>
+      <c r="F110" t="n">
+        <v>1</v>
+      </c>
+      <c r="G110" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2322,6 +2986,12 @@
         <v>9</v>
       </c>
       <c r="E111" t="n">
+        <v>1</v>
+      </c>
+      <c r="F111" t="n">
+        <v>1</v>
+      </c>
+      <c r="G111" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2339,6 +3009,12 @@
         <v>7</v>
       </c>
       <c r="E112" t="n">
+        <v>7</v>
+      </c>
+      <c r="F112" t="n">
+        <v>1</v>
+      </c>
+      <c r="G112" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2356,6 +3032,12 @@
         <v>9</v>
       </c>
       <c r="E113" t="n">
+        <v>4</v>
+      </c>
+      <c r="F113" t="n">
+        <v>4</v>
+      </c>
+      <c r="G113" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2373,6 +3055,12 @@
         <v>7</v>
       </c>
       <c r="E114" t="n">
+        <v>3</v>
+      </c>
+      <c r="F114" t="n">
+        <v>1</v>
+      </c>
+      <c r="G114" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2390,6 +3078,12 @@
         <v>7</v>
       </c>
       <c r="E115" t="n">
+        <v>1</v>
+      </c>
+      <c r="F115" t="n">
+        <v>2</v>
+      </c>
+      <c r="G115" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2407,6 +3101,12 @@
         <v>9</v>
       </c>
       <c r="E116" t="n">
+        <v>3</v>
+      </c>
+      <c r="F116" t="n">
+        <v>0</v>
+      </c>
+      <c r="G116" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2424,6 +3124,12 @@
         <v>7</v>
       </c>
       <c r="E117" t="n">
+        <v>1</v>
+      </c>
+      <c r="F117" t="n">
+        <v>0</v>
+      </c>
+      <c r="G117" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2441,6 +3147,12 @@
         <v>7</v>
       </c>
       <c r="E118" t="n">
+        <v>2</v>
+      </c>
+      <c r="F118" t="n">
+        <v>1</v>
+      </c>
+      <c r="G118" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2458,6 +3170,12 @@
         <v>9</v>
       </c>
       <c r="E119" t="n">
+        <v>8</v>
+      </c>
+      <c r="F119" t="n">
+        <v>0</v>
+      </c>
+      <c r="G119" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2475,6 +3193,12 @@
         <v>7</v>
       </c>
       <c r="E120" t="n">
+        <v>1</v>
+      </c>
+      <c r="F120" t="n">
+        <v>0</v>
+      </c>
+      <c r="G120" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2492,6 +3216,12 @@
         <v>7</v>
       </c>
       <c r="E121" t="n">
+        <v>0</v>
+      </c>
+      <c r="F121" t="n">
+        <v>2</v>
+      </c>
+      <c r="G121" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2509,6 +3239,12 @@
         <v>7</v>
       </c>
       <c r="E122" t="n">
+        <v>3</v>
+      </c>
+      <c r="F122" t="n">
+        <v>1</v>
+      </c>
+      <c r="G122" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2526,6 +3262,12 @@
         <v>9</v>
       </c>
       <c r="E123" t="n">
+        <v>1</v>
+      </c>
+      <c r="F123" t="n">
+        <v>0</v>
+      </c>
+      <c r="G123" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2543,6 +3285,12 @@
         <v>7</v>
       </c>
       <c r="E124" t="n">
+        <v>2</v>
+      </c>
+      <c r="F124" t="n">
+        <v>0</v>
+      </c>
+      <c r="G124" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2560,6 +3308,12 @@
         <v>9</v>
       </c>
       <c r="E125" t="n">
+        <v>10</v>
+      </c>
+      <c r="F125" t="n">
+        <v>1</v>
+      </c>
+      <c r="G125" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2577,6 +3331,12 @@
         <v>7</v>
       </c>
       <c r="E126" t="n">
+        <v>4</v>
+      </c>
+      <c r="F126" t="n">
+        <v>2</v>
+      </c>
+      <c r="G126" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2594,6 +3354,12 @@
         <v>7</v>
       </c>
       <c r="E127" t="n">
+        <v>2</v>
+      </c>
+      <c r="F127" t="n">
+        <v>0</v>
+      </c>
+      <c r="G127" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2611,6 +3377,12 @@
         <v>9</v>
       </c>
       <c r="E128" t="n">
+        <v>1</v>
+      </c>
+      <c r="F128" t="n">
+        <v>0</v>
+      </c>
+      <c r="G128" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2628,6 +3400,12 @@
         <v>7</v>
       </c>
       <c r="E129" t="n">
+        <v>1</v>
+      </c>
+      <c r="F129" t="n">
+        <v>3</v>
+      </c>
+      <c r="G129" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2645,6 +3423,12 @@
         <v>9</v>
       </c>
       <c r="E130" t="n">
+        <v>2</v>
+      </c>
+      <c r="F130" t="n">
+        <v>1</v>
+      </c>
+      <c r="G130" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2662,6 +3446,12 @@
         <v>7</v>
       </c>
       <c r="E131" t="n">
+        <v>3</v>
+      </c>
+      <c r="F131" t="n">
+        <v>0</v>
+      </c>
+      <c r="G131" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2679,6 +3469,12 @@
         <v>7</v>
       </c>
       <c r="E132" t="n">
+        <v>13</v>
+      </c>
+      <c r="F132" t="n">
+        <v>4</v>
+      </c>
+      <c r="G132" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2696,6 +3492,12 @@
         <v>9</v>
       </c>
       <c r="E133" t="n">
+        <v>12</v>
+      </c>
+      <c r="F133" t="n">
+        <v>1</v>
+      </c>
+      <c r="G133" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2713,6 +3515,12 @@
         <v>7</v>
       </c>
       <c r="E134" t="n">
+        <v>1</v>
+      </c>
+      <c r="F134" t="n">
+        <v>0</v>
+      </c>
+      <c r="G134" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2730,6 +3538,12 @@
         <v>9</v>
       </c>
       <c r="E135" t="n">
+        <v>3</v>
+      </c>
+      <c r="F135" t="n">
+        <v>1</v>
+      </c>
+      <c r="G135" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2747,6 +3561,12 @@
         <v>7</v>
       </c>
       <c r="E136" t="n">
+        <v>3</v>
+      </c>
+      <c r="F136" t="n">
+        <v>0</v>
+      </c>
+      <c r="G136" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2764,6 +3584,12 @@
         <v>9</v>
       </c>
       <c r="E137" t="n">
+        <v>19</v>
+      </c>
+      <c r="F137" t="n">
+        <v>2</v>
+      </c>
+      <c r="G137" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2781,6 +3607,12 @@
         <v>7</v>
       </c>
       <c r="E138" t="n">
+        <v>0</v>
+      </c>
+      <c r="F138" t="n">
+        <v>0</v>
+      </c>
+      <c r="G138" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2798,6 +3630,12 @@
         <v>9</v>
       </c>
       <c r="E139" t="n">
+        <v>1</v>
+      </c>
+      <c r="F139" t="n">
+        <v>0</v>
+      </c>
+      <c r="G139" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2815,6 +3653,12 @@
         <v>7</v>
       </c>
       <c r="E140" t="n">
+        <v>8</v>
+      </c>
+      <c r="F140" t="n">
+        <v>2</v>
+      </c>
+      <c r="G140" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2832,6 +3676,12 @@
         <v>7</v>
       </c>
       <c r="E141" t="n">
+        <v>4</v>
+      </c>
+      <c r="F141" t="n">
+        <v>1</v>
+      </c>
+      <c r="G141" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2849,6 +3699,12 @@
         <v>9</v>
       </c>
       <c r="E142" t="n">
+        <v>3</v>
+      </c>
+      <c r="F142" t="n">
+        <v>0</v>
+      </c>
+      <c r="G142" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2866,6 +3722,12 @@
         <v>7</v>
       </c>
       <c r="E143" t="n">
+        <v>7</v>
+      </c>
+      <c r="F143" t="n">
+        <v>1</v>
+      </c>
+      <c r="G143" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2883,6 +3745,12 @@
         <v>9</v>
       </c>
       <c r="E144" t="n">
+        <v>5</v>
+      </c>
+      <c r="F144" t="n">
+        <v>0</v>
+      </c>
+      <c r="G144" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2900,6 +3768,12 @@
         <v>9</v>
       </c>
       <c r="E145" t="n">
+        <v>35</v>
+      </c>
+      <c r="F145" t="n">
+        <v>4</v>
+      </c>
+      <c r="G145" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2917,6 +3791,12 @@
         <v>7</v>
       </c>
       <c r="E146" t="n">
+        <v>6</v>
+      </c>
+      <c r="F146" t="n">
+        <v>1</v>
+      </c>
+      <c r="G146" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2934,6 +3814,12 @@
         <v>9</v>
       </c>
       <c r="E147" t="n">
+        <v>6</v>
+      </c>
+      <c r="F147" t="n">
+        <v>0</v>
+      </c>
+      <c r="G147" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2951,6 +3837,12 @@
         <v>7</v>
       </c>
       <c r="E148" t="n">
+        <v>8</v>
+      </c>
+      <c r="F148" t="n">
+        <v>1</v>
+      </c>
+      <c r="G148" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2968,6 +3860,12 @@
         <v>7</v>
       </c>
       <c r="E149" t="n">
+        <v>1</v>
+      </c>
+      <c r="F149" t="n">
+        <v>2</v>
+      </c>
+      <c r="G149" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -2985,6 +3883,12 @@
         <v>9</v>
       </c>
       <c r="E150" t="n">
+        <v>8</v>
+      </c>
+      <c r="F150" t="n">
+        <v>0</v>
+      </c>
+      <c r="G150" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3002,6 +3906,12 @@
         <v>7</v>
       </c>
       <c r="E151" t="n">
+        <v>17</v>
+      </c>
+      <c r="F151" t="n">
+        <v>5</v>
+      </c>
+      <c r="G151" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3019,6 +3929,12 @@
         <v>9</v>
       </c>
       <c r="E152" t="n">
+        <v>17</v>
+      </c>
+      <c r="F152" t="n">
+        <v>8</v>
+      </c>
+      <c r="G152" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3036,6 +3952,12 @@
         <v>7</v>
       </c>
       <c r="E153" t="n">
+        <v>1</v>
+      </c>
+      <c r="F153" t="n">
+        <v>0</v>
+      </c>
+      <c r="G153" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3053,6 +3975,12 @@
         <v>9</v>
       </c>
       <c r="E154" t="n">
+        <v>1</v>
+      </c>
+      <c r="F154" t="n">
+        <v>0</v>
+      </c>
+      <c r="G154" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3070,6 +3998,12 @@
         <v>9</v>
       </c>
       <c r="E155" t="n">
+        <v>6</v>
+      </c>
+      <c r="F155" t="n">
+        <v>3</v>
+      </c>
+      <c r="G155" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3087,6 +4021,12 @@
         <v>7</v>
       </c>
       <c r="E156" t="n">
+        <v>1</v>
+      </c>
+      <c r="F156" t="n">
+        <v>0</v>
+      </c>
+      <c r="G156" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3104,6 +4044,12 @@
         <v>9</v>
       </c>
       <c r="E157" t="n">
+        <v>5</v>
+      </c>
+      <c r="F157" t="n">
+        <v>1</v>
+      </c>
+      <c r="G157" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3121,6 +4067,12 @@
         <v>7</v>
       </c>
       <c r="E158" t="n">
+        <v>3</v>
+      </c>
+      <c r="F158" t="n">
+        <v>1</v>
+      </c>
+      <c r="G158" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3138,6 +4090,12 @@
         <v>9</v>
       </c>
       <c r="E159" t="n">
+        <v>1</v>
+      </c>
+      <c r="F159" t="n">
+        <v>0</v>
+      </c>
+      <c r="G159" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3155,6 +4113,12 @@
         <v>7</v>
       </c>
       <c r="E160" t="n">
+        <v>6</v>
+      </c>
+      <c r="F160" t="n">
+        <v>0</v>
+      </c>
+      <c r="G160" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3172,6 +4136,12 @@
         <v>7</v>
       </c>
       <c r="E161" t="n">
+        <v>13</v>
+      </c>
+      <c r="F161" t="n">
+        <v>0</v>
+      </c>
+      <c r="G161" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3189,6 +4159,12 @@
         <v>9</v>
       </c>
       <c r="E162" t="n">
+        <v>17</v>
+      </c>
+      <c r="F162" t="n">
+        <v>3</v>
+      </c>
+      <c r="G162" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3206,6 +4182,12 @@
         <v>7</v>
       </c>
       <c r="E163" t="n">
+        <v>23</v>
+      </c>
+      <c r="F163" t="n">
+        <v>7</v>
+      </c>
+      <c r="G163" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3223,6 +4205,12 @@
         <v>9</v>
       </c>
       <c r="E164" t="n">
+        <v>6</v>
+      </c>
+      <c r="F164" t="n">
+        <v>1</v>
+      </c>
+      <c r="G164" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3240,6 +4228,12 @@
         <v>7</v>
       </c>
       <c r="E165" t="n">
+        <v>4</v>
+      </c>
+      <c r="F165" t="n">
+        <v>0</v>
+      </c>
+      <c r="G165" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3257,6 +4251,12 @@
         <v>9</v>
       </c>
       <c r="E166" t="n">
+        <v>2</v>
+      </c>
+      <c r="F166" t="n">
+        <v>0</v>
+      </c>
+      <c r="G166" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3274,6 +4274,12 @@
         <v>7</v>
       </c>
       <c r="E167" t="n">
+        <v>1</v>
+      </c>
+      <c r="F167" t="n">
+        <v>0</v>
+      </c>
+      <c r="G167" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3291,6 +4297,12 @@
         <v>9</v>
       </c>
       <c r="E168" t="n">
+        <v>5</v>
+      </c>
+      <c r="F168" t="n">
+        <v>0</v>
+      </c>
+      <c r="G168" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3308,6 +4320,12 @@
         <v>7</v>
       </c>
       <c r="E169" t="n">
+        <v>1</v>
+      </c>
+      <c r="F169" t="n">
+        <v>0</v>
+      </c>
+      <c r="G169" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3325,6 +4343,12 @@
         <v>9</v>
       </c>
       <c r="E170" t="n">
+        <v>4</v>
+      </c>
+      <c r="F170" t="n">
+        <v>2</v>
+      </c>
+      <c r="G170" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3342,6 +4366,12 @@
         <v>7</v>
       </c>
       <c r="E171" t="n">
+        <v>0</v>
+      </c>
+      <c r="F171" t="n">
+        <v>0</v>
+      </c>
+      <c r="G171" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3359,6 +4389,12 @@
         <v>7</v>
       </c>
       <c r="E172" t="n">
+        <v>2</v>
+      </c>
+      <c r="F172" t="n">
+        <v>1</v>
+      </c>
+      <c r="G172" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3376,6 +4412,12 @@
         <v>7</v>
       </c>
       <c r="E173" t="n">
+        <v>4</v>
+      </c>
+      <c r="F173" t="n">
+        <v>1</v>
+      </c>
+      <c r="G173" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3393,6 +4435,12 @@
         <v>7</v>
       </c>
       <c r="E174" t="n">
+        <v>2</v>
+      </c>
+      <c r="F174" t="n">
+        <v>0</v>
+      </c>
+      <c r="G174" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3410,6 +4458,12 @@
         <v>7</v>
       </c>
       <c r="E175" t="n">
+        <v>5</v>
+      </c>
+      <c r="F175" t="n">
+        <v>2</v>
+      </c>
+      <c r="G175" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3427,6 +4481,12 @@
         <v>9</v>
       </c>
       <c r="E176" t="n">
+        <v>8</v>
+      </c>
+      <c r="F176" t="n">
+        <v>1</v>
+      </c>
+      <c r="G176" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3444,6 +4504,12 @@
         <v>7</v>
       </c>
       <c r="E177" t="n">
+        <v>0</v>
+      </c>
+      <c r="F177" t="n">
+        <v>0</v>
+      </c>
+      <c r="G177" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3461,6 +4527,12 @@
         <v>9</v>
       </c>
       <c r="E178" t="n">
+        <v>4</v>
+      </c>
+      <c r="F178" t="n">
+        <v>0</v>
+      </c>
+      <c r="G178" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3478,6 +4550,12 @@
         <v>7</v>
       </c>
       <c r="E179" t="n">
+        <v>5</v>
+      </c>
+      <c r="F179" t="n">
+        <v>3</v>
+      </c>
+      <c r="G179" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3495,6 +4573,12 @@
         <v>7</v>
       </c>
       <c r="E180" t="n">
+        <v>0</v>
+      </c>
+      <c r="F180" t="n">
+        <v>1</v>
+      </c>
+      <c r="G180" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3512,6 +4596,12 @@
         <v>7</v>
       </c>
       <c r="E181" t="n">
+        <v>0</v>
+      </c>
+      <c r="F181" t="n">
+        <v>0</v>
+      </c>
+      <c r="G181" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3529,6 +4619,12 @@
         <v>7</v>
       </c>
       <c r="E182" t="n">
+        <v>1</v>
+      </c>
+      <c r="F182" t="n">
+        <v>0</v>
+      </c>
+      <c r="G182" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3546,6 +4642,12 @@
         <v>7</v>
       </c>
       <c r="E183" t="n">
+        <v>0</v>
+      </c>
+      <c r="F183" t="n">
+        <v>1</v>
+      </c>
+      <c r="G183" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3563,6 +4665,12 @@
         <v>7</v>
       </c>
       <c r="E184" t="n">
+        <v>1</v>
+      </c>
+      <c r="F184" t="n">
+        <v>1</v>
+      </c>
+      <c r="G184" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3580,6 +4688,12 @@
         <v>9</v>
       </c>
       <c r="E185" t="n">
+        <v>7</v>
+      </c>
+      <c r="F185" t="n">
+        <v>0</v>
+      </c>
+      <c r="G185" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3597,6 +4711,12 @@
         <v>7</v>
       </c>
       <c r="E186" t="n">
+        <v>3</v>
+      </c>
+      <c r="F186" t="n">
+        <v>4</v>
+      </c>
+      <c r="G186" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3614,6 +4734,12 @@
         <v>9</v>
       </c>
       <c r="E187" t="n">
+        <v>7</v>
+      </c>
+      <c r="F187" t="n">
+        <v>0</v>
+      </c>
+      <c r="G187" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3631,6 +4757,12 @@
         <v>9</v>
       </c>
       <c r="E188" t="n">
+        <v>7</v>
+      </c>
+      <c r="F188" t="n">
+        <v>0</v>
+      </c>
+      <c r="G188" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3648,6 +4780,12 @@
         <v>7</v>
       </c>
       <c r="E189" t="n">
+        <v>0</v>
+      </c>
+      <c r="F189" t="n">
+        <v>0</v>
+      </c>
+      <c r="G189" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3665,6 +4803,12 @@
         <v>9</v>
       </c>
       <c r="E190" t="n">
+        <v>0</v>
+      </c>
+      <c r="F190" t="n">
+        <v>0</v>
+      </c>
+      <c r="G190" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3682,6 +4826,12 @@
         <v>7</v>
       </c>
       <c r="E191" t="n">
+        <v>4</v>
+      </c>
+      <c r="F191" t="n">
+        <v>0</v>
+      </c>
+      <c r="G191" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3699,6 +4849,12 @@
         <v>7</v>
       </c>
       <c r="E192" t="n">
+        <v>4</v>
+      </c>
+      <c r="F192" t="n">
+        <v>2</v>
+      </c>
+      <c r="G192" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3716,6 +4872,12 @@
         <v>9</v>
       </c>
       <c r="E193" t="n">
+        <v>10</v>
+      </c>
+      <c r="F193" t="n">
+        <v>3</v>
+      </c>
+      <c r="G193" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3733,6 +4895,12 @@
         <v>7</v>
       </c>
       <c r="E194" t="n">
+        <v>8</v>
+      </c>
+      <c r="F194" t="n">
+        <v>1</v>
+      </c>
+      <c r="G194" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3750,6 +4918,12 @@
         <v>9</v>
       </c>
       <c r="E195" t="n">
+        <v>8</v>
+      </c>
+      <c r="F195" t="n">
+        <v>1</v>
+      </c>
+      <c r="G195" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3767,6 +4941,12 @@
         <v>7</v>
       </c>
       <c r="E196" t="n">
+        <v>1</v>
+      </c>
+      <c r="F196" t="n">
+        <v>0</v>
+      </c>
+      <c r="G196" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3784,6 +4964,12 @@
         <v>7</v>
       </c>
       <c r="E197" t="n">
+        <v>1</v>
+      </c>
+      <c r="F197" t="n">
+        <v>0</v>
+      </c>
+      <c r="G197" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3801,6 +4987,12 @@
         <v>7</v>
       </c>
       <c r="E198" t="n">
+        <v>2</v>
+      </c>
+      <c r="F198" t="n">
+        <v>1</v>
+      </c>
+      <c r="G198" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3818,6 +5010,12 @@
         <v>7</v>
       </c>
       <c r="E199" t="n">
+        <v>3</v>
+      </c>
+      <c r="F199" t="n">
+        <v>0</v>
+      </c>
+      <c r="G199" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3835,6 +5033,12 @@
         <v>7</v>
       </c>
       <c r="E200" t="n">
+        <v>7</v>
+      </c>
+      <c r="F200" t="n">
+        <v>0</v>
+      </c>
+      <c r="G200" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3852,6 +5056,12 @@
         <v>7</v>
       </c>
       <c r="E201" t="n">
+        <v>2</v>
+      </c>
+      <c r="F201" t="n">
+        <v>0</v>
+      </c>
+      <c r="G201" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3869,6 +5079,12 @@
         <v>9</v>
       </c>
       <c r="E202" t="n">
+        <v>7</v>
+      </c>
+      <c r="F202" t="n">
+        <v>1</v>
+      </c>
+      <c r="G202" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3886,6 +5102,12 @@
         <v>7</v>
       </c>
       <c r="E203" t="n">
+        <v>0</v>
+      </c>
+      <c r="F203" t="n">
+        <v>0</v>
+      </c>
+      <c r="G203" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3903,6 +5125,12 @@
         <v>7</v>
       </c>
       <c r="E204" t="n">
+        <v>3</v>
+      </c>
+      <c r="F204" t="n">
+        <v>3</v>
+      </c>
+      <c r="G204" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3920,6 +5148,12 @@
         <v>7</v>
       </c>
       <c r="E205" t="n">
+        <v>9</v>
+      </c>
+      <c r="F205" t="n">
+        <v>0</v>
+      </c>
+      <c r="G205" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3937,6 +5171,12 @@
         <v>7</v>
       </c>
       <c r="E206" t="n">
+        <v>1</v>
+      </c>
+      <c r="F206" t="n">
+        <v>0</v>
+      </c>
+      <c r="G206" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3954,6 +5194,12 @@
         <v>9</v>
       </c>
       <c r="E207" t="n">
+        <v>4</v>
+      </c>
+      <c r="F207" t="n">
+        <v>0</v>
+      </c>
+      <c r="G207" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3971,6 +5217,12 @@
         <v>7</v>
       </c>
       <c r="E208" t="n">
+        <v>30</v>
+      </c>
+      <c r="F208" t="n">
+        <v>4</v>
+      </c>
+      <c r="G208" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -3988,6 +5240,12 @@
         <v>9</v>
       </c>
       <c r="E209" t="n">
+        <v>25</v>
+      </c>
+      <c r="F209" t="n">
+        <v>0</v>
+      </c>
+      <c r="G209" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4005,6 +5263,12 @@
         <v>7</v>
       </c>
       <c r="E210" t="n">
+        <v>1</v>
+      </c>
+      <c r="F210" t="n">
+        <v>4</v>
+      </c>
+      <c r="G210" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4022,6 +5286,12 @@
         <v>9</v>
       </c>
       <c r="E211" t="n">
+        <v>5</v>
+      </c>
+      <c r="F211" t="n">
+        <v>0</v>
+      </c>
+      <c r="G211" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4039,6 +5309,12 @@
         <v>7</v>
       </c>
       <c r="E212" t="n">
+        <v>1</v>
+      </c>
+      <c r="F212" t="n">
+        <v>0</v>
+      </c>
+      <c r="G212" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4056,6 +5332,12 @@
         <v>7</v>
       </c>
       <c r="E213" t="n">
+        <v>8</v>
+      </c>
+      <c r="F213" t="n">
+        <v>0</v>
+      </c>
+      <c r="G213" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4073,6 +5355,12 @@
         <v>9</v>
       </c>
       <c r="E214" t="n">
+        <v>11</v>
+      </c>
+      <c r="F214" t="n">
+        <v>2</v>
+      </c>
+      <c r="G214" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4090,6 +5378,12 @@
         <v>9</v>
       </c>
       <c r="E215" t="n">
+        <v>1</v>
+      </c>
+      <c r="F215" t="n">
+        <v>0</v>
+      </c>
+      <c r="G215" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4107,6 +5401,12 @@
         <v>7</v>
       </c>
       <c r="E216" t="n">
+        <v>2</v>
+      </c>
+      <c r="F216" t="n">
+        <v>0</v>
+      </c>
+      <c r="G216" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4124,6 +5424,12 @@
         <v>7</v>
       </c>
       <c r="E217" t="n">
+        <v>1</v>
+      </c>
+      <c r="F217" t="n">
+        <v>0</v>
+      </c>
+      <c r="G217" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4141,6 +5447,12 @@
         <v>9</v>
       </c>
       <c r="E218" t="n">
+        <v>2</v>
+      </c>
+      <c r="F218" t="n">
+        <v>0</v>
+      </c>
+      <c r="G218" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4158,6 +5470,12 @@
         <v>7</v>
       </c>
       <c r="E219" t="n">
+        <v>1</v>
+      </c>
+      <c r="F219" t="n">
+        <v>0</v>
+      </c>
+      <c r="G219" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4175,6 +5493,12 @@
         <v>9</v>
       </c>
       <c r="E220" t="n">
+        <v>2</v>
+      </c>
+      <c r="F220" t="n">
+        <v>2</v>
+      </c>
+      <c r="G220" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4192,6 +5516,12 @@
         <v>7</v>
       </c>
       <c r="E221" t="n">
+        <v>6</v>
+      </c>
+      <c r="F221" t="n">
+        <v>1</v>
+      </c>
+      <c r="G221" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4209,6 +5539,12 @@
         <v>9</v>
       </c>
       <c r="E222" t="n">
+        <v>3</v>
+      </c>
+      <c r="F222" t="n">
+        <v>1</v>
+      </c>
+      <c r="G222" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4226,6 +5562,12 @@
         <v>9</v>
       </c>
       <c r="E223" t="n">
+        <v>5</v>
+      </c>
+      <c r="F223" t="n">
+        <v>0</v>
+      </c>
+      <c r="G223" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4243,6 +5585,12 @@
         <v>9</v>
       </c>
       <c r="E224" t="n">
+        <v>2</v>
+      </c>
+      <c r="F224" t="n">
+        <v>1</v>
+      </c>
+      <c r="G224" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4260,6 +5608,12 @@
         <v>7</v>
       </c>
       <c r="E225" t="n">
+        <v>5</v>
+      </c>
+      <c r="F225" t="n">
+        <v>2</v>
+      </c>
+      <c r="G225" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4277,6 +5631,12 @@
         <v>7</v>
       </c>
       <c r="E226" t="n">
+        <v>1</v>
+      </c>
+      <c r="F226" t="n">
+        <v>1</v>
+      </c>
+      <c r="G226" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4294,6 +5654,12 @@
         <v>7</v>
       </c>
       <c r="E227" t="n">
+        <v>1</v>
+      </c>
+      <c r="F227" t="n">
+        <v>0</v>
+      </c>
+      <c r="G227" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4311,6 +5677,12 @@
         <v>9</v>
       </c>
       <c r="E228" t="n">
+        <v>2</v>
+      </c>
+      <c r="F228" t="n">
+        <v>0</v>
+      </c>
+      <c r="G228" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4328,6 +5700,12 @@
         <v>7</v>
       </c>
       <c r="E229" t="n">
+        <v>2</v>
+      </c>
+      <c r="F229" t="n">
+        <v>0</v>
+      </c>
+      <c r="G229" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4345,6 +5723,12 @@
         <v>7</v>
       </c>
       <c r="E230" t="n">
+        <v>4</v>
+      </c>
+      <c r="F230" t="n">
+        <v>1</v>
+      </c>
+      <c r="G230" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4362,6 +5746,12 @@
         <v>9</v>
       </c>
       <c r="E231" t="n">
+        <v>7</v>
+      </c>
+      <c r="F231" t="n">
+        <v>2</v>
+      </c>
+      <c r="G231" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4379,6 +5769,12 @@
         <v>7</v>
       </c>
       <c r="E232" t="n">
+        <v>12</v>
+      </c>
+      <c r="F232" t="n">
+        <v>0</v>
+      </c>
+      <c r="G232" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4396,6 +5792,12 @@
         <v>9</v>
       </c>
       <c r="E233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F233" t="n">
+        <v>1</v>
+      </c>
+      <c r="G233" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4413,6 +5815,12 @@
         <v>9</v>
       </c>
       <c r="E234" t="n">
+        <v>1</v>
+      </c>
+      <c r="F234" t="n">
+        <v>0</v>
+      </c>
+      <c r="G234" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4430,6 +5838,12 @@
         <v>7</v>
       </c>
       <c r="E235" t="n">
+        <v>2</v>
+      </c>
+      <c r="F235" t="n">
+        <v>2</v>
+      </c>
+      <c r="G235" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4447,6 +5861,12 @@
         <v>7</v>
       </c>
       <c r="E236" t="n">
+        <v>1</v>
+      </c>
+      <c r="F236" t="n">
+        <v>0</v>
+      </c>
+      <c r="G236" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4464,6 +5884,12 @@
         <v>7</v>
       </c>
       <c r="E237" t="n">
+        <v>3</v>
+      </c>
+      <c r="F237" t="n">
+        <v>1</v>
+      </c>
+      <c r="G237" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4481,6 +5907,12 @@
         <v>9</v>
       </c>
       <c r="E238" t="n">
+        <v>1</v>
+      </c>
+      <c r="F238" t="n">
+        <v>0</v>
+      </c>
+      <c r="G238" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4498,6 +5930,12 @@
         <v>9</v>
       </c>
       <c r="E239" t="n">
+        <v>6</v>
+      </c>
+      <c r="F239" t="n">
+        <v>1</v>
+      </c>
+      <c r="G239" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4515,6 +5953,12 @@
         <v>7</v>
       </c>
       <c r="E240" t="n">
+        <v>7</v>
+      </c>
+      <c r="F240" t="n">
+        <v>1</v>
+      </c>
+      <c r="G240" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4532,6 +5976,12 @@
         <v>9</v>
       </c>
       <c r="E241" t="n">
+        <v>5</v>
+      </c>
+      <c r="F241" t="n">
+        <v>1</v>
+      </c>
+      <c r="G241" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4549,6 +5999,12 @@
         <v>9</v>
       </c>
       <c r="E242" t="n">
+        <v>1</v>
+      </c>
+      <c r="F242" t="n">
+        <v>0</v>
+      </c>
+      <c r="G242" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4566,6 +6022,12 @@
         <v>7</v>
       </c>
       <c r="E243" t="n">
+        <v>0</v>
+      </c>
+      <c r="F243" t="n">
+        <v>0</v>
+      </c>
+      <c r="G243" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4583,6 +6045,12 @@
         <v>9</v>
       </c>
       <c r="E244" t="n">
+        <v>4</v>
+      </c>
+      <c r="F244" t="n">
+        <v>0</v>
+      </c>
+      <c r="G244" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4600,6 +6068,12 @@
         <v>7</v>
       </c>
       <c r="E245" t="n">
+        <v>2</v>
+      </c>
+      <c r="F245" t="n">
+        <v>0</v>
+      </c>
+      <c r="G245" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4617,6 +6091,12 @@
         <v>9</v>
       </c>
       <c r="E246" t="n">
+        <v>2</v>
+      </c>
+      <c r="F246" t="n">
+        <v>0</v>
+      </c>
+      <c r="G246" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4634,6 +6114,12 @@
         <v>7</v>
       </c>
       <c r="E247" t="n">
+        <v>2</v>
+      </c>
+      <c r="F247" t="n">
+        <v>0</v>
+      </c>
+      <c r="G247" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4651,6 +6137,12 @@
         <v>7</v>
       </c>
       <c r="E248" t="n">
+        <v>1</v>
+      </c>
+      <c r="F248" t="n">
+        <v>0</v>
+      </c>
+      <c r="G248" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4668,6 +6160,12 @@
         <v>9</v>
       </c>
       <c r="E249" t="n">
+        <v>4</v>
+      </c>
+      <c r="F249" t="n">
+        <v>0</v>
+      </c>
+      <c r="G249" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4685,6 +6183,12 @@
         <v>7</v>
       </c>
       <c r="E250" t="n">
+        <v>13</v>
+      </c>
+      <c r="F250" t="n">
+        <v>1</v>
+      </c>
+      <c r="G250" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4702,6 +6206,12 @@
         <v>9</v>
       </c>
       <c r="E251" t="n">
+        <v>9</v>
+      </c>
+      <c r="F251" t="n">
+        <v>1</v>
+      </c>
+      <c r="G251" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4719,6 +6229,12 @@
         <v>9</v>
       </c>
       <c r="E252" t="n">
+        <v>0</v>
+      </c>
+      <c r="F252" t="n">
+        <v>1</v>
+      </c>
+      <c r="G252" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4736,6 +6252,12 @@
         <v>7</v>
       </c>
       <c r="E253" t="n">
+        <v>2</v>
+      </c>
+      <c r="F253" t="n">
+        <v>2</v>
+      </c>
+      <c r="G253" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4753,6 +6275,12 @@
         <v>9</v>
       </c>
       <c r="E254" t="n">
+        <v>5</v>
+      </c>
+      <c r="F254" t="n">
+        <v>3</v>
+      </c>
+      <c r="G254" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4770,6 +6298,12 @@
         <v>7</v>
       </c>
       <c r="E255" t="n">
+        <v>3</v>
+      </c>
+      <c r="F255" t="n">
+        <v>2</v>
+      </c>
+      <c r="G255" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4787,6 +6321,12 @@
         <v>9</v>
       </c>
       <c r="E256" t="n">
+        <v>0</v>
+      </c>
+      <c r="F256" t="n">
+        <v>1</v>
+      </c>
+      <c r="G256" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4804,6 +6344,12 @@
         <v>9</v>
       </c>
       <c r="E257" t="n">
+        <v>3</v>
+      </c>
+      <c r="F257" t="n">
+        <v>0</v>
+      </c>
+      <c r="G257" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4821,6 +6367,12 @@
         <v>7</v>
       </c>
       <c r="E258" t="n">
+        <v>7</v>
+      </c>
+      <c r="F258" t="n">
+        <v>2</v>
+      </c>
+      <c r="G258" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4838,6 +6390,12 @@
         <v>9</v>
       </c>
       <c r="E259" t="n">
+        <v>14</v>
+      </c>
+      <c r="F259" t="n">
+        <v>2</v>
+      </c>
+      <c r="G259" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4855,6 +6413,12 @@
         <v>7</v>
       </c>
       <c r="E260" t="n">
+        <v>0</v>
+      </c>
+      <c r="F260" t="n">
+        <v>0</v>
+      </c>
+      <c r="G260" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4872,6 +6436,12 @@
         <v>7</v>
       </c>
       <c r="E261" t="n">
+        <v>1</v>
+      </c>
+      <c r="F261" t="n">
+        <v>0</v>
+      </c>
+      <c r="G261" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4889,6 +6459,12 @@
         <v>7</v>
       </c>
       <c r="E262" t="n">
+        <v>4</v>
+      </c>
+      <c r="F262" t="n">
+        <v>1</v>
+      </c>
+      <c r="G262" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4906,6 +6482,12 @@
         <v>9</v>
       </c>
       <c r="E263" t="n">
+        <v>4</v>
+      </c>
+      <c r="F263" t="n">
+        <v>0</v>
+      </c>
+      <c r="G263" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4923,6 +6505,12 @@
         <v>7</v>
       </c>
       <c r="E264" t="n">
+        <v>4</v>
+      </c>
+      <c r="F264" t="n">
+        <v>3</v>
+      </c>
+      <c r="G264" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4940,6 +6528,12 @@
         <v>7</v>
       </c>
       <c r="E265" t="n">
+        <v>3</v>
+      </c>
+      <c r="F265" t="n">
+        <v>0</v>
+      </c>
+      <c r="G265" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4957,6 +6551,12 @@
         <v>7</v>
       </c>
       <c r="E266" t="n">
+        <v>10</v>
+      </c>
+      <c r="F266" t="n">
+        <v>1</v>
+      </c>
+      <c r="G266" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4974,6 +6574,12 @@
         <v>9</v>
       </c>
       <c r="E267" t="n">
+        <v>10</v>
+      </c>
+      <c r="F267" t="n">
+        <v>0</v>
+      </c>
+      <c r="G267" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4991,6 +6597,12 @@
         <v>7</v>
       </c>
       <c r="E268" t="n">
+        <v>7</v>
+      </c>
+      <c r="F268" t="n">
+        <v>2</v>
+      </c>
+      <c r="G268" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5008,6 +6620,12 @@
         <v>9</v>
       </c>
       <c r="E269" t="n">
+        <v>5</v>
+      </c>
+      <c r="F269" t="n">
+        <v>0</v>
+      </c>
+      <c r="G269" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5025,6 +6643,12 @@
         <v>7</v>
       </c>
       <c r="E270" t="n">
+        <v>3</v>
+      </c>
+      <c r="F270" t="n">
+        <v>0</v>
+      </c>
+      <c r="G270" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5042,6 +6666,12 @@
         <v>9</v>
       </c>
       <c r="E271" t="n">
+        <v>5</v>
+      </c>
+      <c r="F271" t="n">
+        <v>0</v>
+      </c>
+      <c r="G271" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5059,6 +6689,12 @@
         <v>7</v>
       </c>
       <c r="E272" t="n">
+        <v>7</v>
+      </c>
+      <c r="F272" t="n">
+        <v>0</v>
+      </c>
+      <c r="G272" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5076,6 +6712,12 @@
         <v>9</v>
       </c>
       <c r="E273" t="n">
+        <v>20</v>
+      </c>
+      <c r="F273" t="n">
+        <v>2</v>
+      </c>
+      <c r="G273" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5093,6 +6735,12 @@
         <v>9</v>
       </c>
       <c r="E274" t="n">
+        <v>4</v>
+      </c>
+      <c r="F274" t="n">
+        <v>1</v>
+      </c>
+      <c r="G274" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5110,6 +6758,12 @@
         <v>7</v>
       </c>
       <c r="E275" t="n">
+        <v>11</v>
+      </c>
+      <c r="F275" t="n">
+        <v>4</v>
+      </c>
+      <c r="G275" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5127,6 +6781,12 @@
         <v>9</v>
       </c>
       <c r="E276" t="n">
+        <v>15</v>
+      </c>
+      <c r="F276" t="n">
+        <v>0</v>
+      </c>
+      <c r="G276" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5144,6 +6804,12 @@
         <v>9</v>
       </c>
       <c r="E277" t="n">
+        <v>26</v>
+      </c>
+      <c r="F277" t="n">
+        <v>2</v>
+      </c>
+      <c r="G277" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5161,6 +6827,12 @@
         <v>7</v>
       </c>
       <c r="E278" t="n">
+        <v>7</v>
+      </c>
+      <c r="F278" t="n">
+        <v>4</v>
+      </c>
+      <c r="G278" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5178,6 +6850,12 @@
         <v>9</v>
       </c>
       <c r="E279" t="n">
+        <v>7</v>
+      </c>
+      <c r="F279" t="n">
+        <v>0</v>
+      </c>
+      <c r="G279" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5195,6 +6873,12 @@
         <v>7</v>
       </c>
       <c r="E280" t="n">
+        <v>3</v>
+      </c>
+      <c r="F280" t="n">
+        <v>2</v>
+      </c>
+      <c r="G280" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5212,6 +6896,12 @@
         <v>7</v>
       </c>
       <c r="E281" t="n">
+        <v>28</v>
+      </c>
+      <c r="F281" t="n">
+        <v>5</v>
+      </c>
+      <c r="G281" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5229,6 +6919,12 @@
         <v>7</v>
       </c>
       <c r="E282" t="n">
+        <v>10</v>
+      </c>
+      <c r="F282" t="n">
+        <v>1</v>
+      </c>
+      <c r="G282" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5246,6 +6942,12 @@
         <v>7</v>
       </c>
       <c r="E283" t="n">
+        <v>3</v>
+      </c>
+      <c r="F283" t="n">
+        <v>0</v>
+      </c>
+      <c r="G283" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5263,6 +6965,12 @@
         <v>7</v>
       </c>
       <c r="E284" t="n">
+        <v>1</v>
+      </c>
+      <c r="F284" t="n">
+        <v>1</v>
+      </c>
+      <c r="G284" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5280,6 +6988,12 @@
         <v>7</v>
       </c>
       <c r="E285" t="n">
+        <v>4</v>
+      </c>
+      <c r="F285" t="n">
+        <v>0</v>
+      </c>
+      <c r="G285" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5297,6 +7011,12 @@
         <v>7</v>
       </c>
       <c r="E286" t="n">
+        <v>12</v>
+      </c>
+      <c r="F286" t="n">
+        <v>2</v>
+      </c>
+      <c r="G286" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5314,6 +7034,12 @@
         <v>9</v>
       </c>
       <c r="E287" t="n">
+        <v>7</v>
+      </c>
+      <c r="F287" t="n">
+        <v>3</v>
+      </c>
+      <c r="G287" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5331,6 +7057,12 @@
         <v>7</v>
       </c>
       <c r="E288" t="n">
+        <v>4</v>
+      </c>
+      <c r="F288" t="n">
+        <v>0</v>
+      </c>
+      <c r="G288" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5348,6 +7080,12 @@
         <v>9</v>
       </c>
       <c r="E289" t="n">
+        <v>3</v>
+      </c>
+      <c r="F289" t="n">
+        <v>0</v>
+      </c>
+      <c r="G289" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5365,6 +7103,12 @@
         <v>9</v>
       </c>
       <c r="E290" t="n">
+        <v>9</v>
+      </c>
+      <c r="F290" t="n">
+        <v>1</v>
+      </c>
+      <c r="G290" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5382,6 +7126,12 @@
         <v>7</v>
       </c>
       <c r="E291" t="n">
+        <v>2</v>
+      </c>
+      <c r="F291" t="n">
+        <v>1</v>
+      </c>
+      <c r="G291" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5399,6 +7149,12 @@
         <v>7</v>
       </c>
       <c r="E292" t="n">
+        <v>2</v>
+      </c>
+      <c r="F292" t="n">
+        <v>1</v>
+      </c>
+      <c r="G292" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5416,6 +7172,12 @@
         <v>9</v>
       </c>
       <c r="E293" t="n">
+        <v>9</v>
+      </c>
+      <c r="F293" t="n">
+        <v>1</v>
+      </c>
+      <c r="G293" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5433,6 +7195,12 @@
         <v>7</v>
       </c>
       <c r="E294" t="n">
+        <v>2</v>
+      </c>
+      <c r="F294" t="n">
+        <v>0</v>
+      </c>
+      <c r="G294" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5450,6 +7218,12 @@
         <v>9</v>
       </c>
       <c r="E295" t="n">
+        <v>2</v>
+      </c>
+      <c r="F295" t="n">
+        <v>0</v>
+      </c>
+      <c r="G295" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5467,6 +7241,12 @@
         <v>7</v>
       </c>
       <c r="E296" t="n">
+        <v>2</v>
+      </c>
+      <c r="F296" t="n">
+        <v>0</v>
+      </c>
+      <c r="G296" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5484,6 +7264,12 @@
         <v>9</v>
       </c>
       <c r="E297" t="n">
+        <v>3</v>
+      </c>
+      <c r="F297" t="n">
+        <v>0</v>
+      </c>
+      <c r="G297" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5501,6 +7287,12 @@
         <v>7</v>
       </c>
       <c r="E298" t="n">
+        <v>6</v>
+      </c>
+      <c r="F298" t="n">
+        <v>2</v>
+      </c>
+      <c r="G298" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5518,6 +7310,12 @@
         <v>9</v>
       </c>
       <c r="E299" t="n">
+        <v>7</v>
+      </c>
+      <c r="F299" t="n">
+        <v>1</v>
+      </c>
+      <c r="G299" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5535,6 +7333,12 @@
         <v>7</v>
       </c>
       <c r="E300" t="n">
+        <v>1</v>
+      </c>
+      <c r="F300" t="n">
+        <v>0</v>
+      </c>
+      <c r="G300" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5552,6 +7356,12 @@
         <v>9</v>
       </c>
       <c r="E301" t="n">
+        <v>3</v>
+      </c>
+      <c r="F301" t="n">
+        <v>0</v>
+      </c>
+      <c r="G301" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5569,6 +7379,12 @@
         <v>7</v>
       </c>
       <c r="E302" t="n">
+        <v>6</v>
+      </c>
+      <c r="F302" t="n">
+        <v>1</v>
+      </c>
+      <c r="G302" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5586,6 +7402,12 @@
         <v>9</v>
       </c>
       <c r="E303" t="n">
+        <v>8</v>
+      </c>
+      <c r="F303" t="n">
+        <v>0</v>
+      </c>
+      <c r="G303" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5603,6 +7425,12 @@
         <v>7</v>
       </c>
       <c r="E304" t="n">
+        <v>0</v>
+      </c>
+      <c r="F304" t="n">
+        <v>1</v>
+      </c>
+      <c r="G304" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5620,6 +7448,12 @@
         <v>9</v>
       </c>
       <c r="E305" t="n">
+        <v>6</v>
+      </c>
+      <c r="F305" t="n">
+        <v>0</v>
+      </c>
+      <c r="G305" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5637,6 +7471,12 @@
         <v>7</v>
       </c>
       <c r="E306" t="n">
+        <v>5</v>
+      </c>
+      <c r="F306" t="n">
+        <v>4</v>
+      </c>
+      <c r="G306" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5654,6 +7494,12 @@
         <v>9</v>
       </c>
       <c r="E307" t="n">
+        <v>4</v>
+      </c>
+      <c r="F307" t="n">
+        <v>1</v>
+      </c>
+      <c r="G307" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5671,6 +7517,12 @@
         <v>7</v>
       </c>
       <c r="E308" t="n">
+        <v>4</v>
+      </c>
+      <c r="F308" t="n">
+        <v>1</v>
+      </c>
+      <c r="G308" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5688,6 +7540,12 @@
         <v>9</v>
       </c>
       <c r="E309" t="n">
+        <v>4</v>
+      </c>
+      <c r="F309" t="n">
+        <v>1</v>
+      </c>
+      <c r="G309" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5705,6 +7563,12 @@
         <v>7</v>
       </c>
       <c r="E310" t="n">
+        <v>2</v>
+      </c>
+      <c r="F310" t="n">
+        <v>1</v>
+      </c>
+      <c r="G310" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5722,6 +7586,12 @@
         <v>7</v>
       </c>
       <c r="E311" t="n">
+        <v>2</v>
+      </c>
+      <c r="F311" t="n">
+        <v>0</v>
+      </c>
+      <c r="G311" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5739,6 +7609,12 @@
         <v>7</v>
       </c>
       <c r="E312" t="n">
+        <v>2</v>
+      </c>
+      <c r="F312" t="n">
+        <v>1</v>
+      </c>
+      <c r="G312" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5756,6 +7632,12 @@
         <v>9</v>
       </c>
       <c r="E313" t="n">
+        <v>7</v>
+      </c>
+      <c r="F313" t="n">
+        <v>3</v>
+      </c>
+      <c r="G313" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5773,6 +7655,12 @@
         <v>7</v>
       </c>
       <c r="E314" t="n">
+        <v>7</v>
+      </c>
+      <c r="F314" t="n">
+        <v>0</v>
+      </c>
+      <c r="G314" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5790,6 +7678,12 @@
         <v>9</v>
       </c>
       <c r="E315" t="n">
+        <v>6</v>
+      </c>
+      <c r="F315" t="n">
+        <v>1</v>
+      </c>
+      <c r="G315" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5807,6 +7701,12 @@
         <v>7</v>
       </c>
       <c r="E316" t="n">
+        <v>0</v>
+      </c>
+      <c r="F316" t="n">
+        <v>0</v>
+      </c>
+      <c r="G316" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5824,6 +7724,12 @@
         <v>9</v>
       </c>
       <c r="E317" t="n">
+        <v>0</v>
+      </c>
+      <c r="F317" t="n">
+        <v>0</v>
+      </c>
+      <c r="G317" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5841,6 +7747,12 @@
         <v>7</v>
       </c>
       <c r="E318" t="n">
+        <v>1</v>
+      </c>
+      <c r="F318" t="n">
+        <v>0</v>
+      </c>
+      <c r="G318" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5858,6 +7770,12 @@
         <v>7</v>
       </c>
       <c r="E319" t="n">
+        <v>7</v>
+      </c>
+      <c r="F319" t="n">
+        <v>3</v>
+      </c>
+      <c r="G319" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5875,6 +7793,12 @@
         <v>9</v>
       </c>
       <c r="E320" t="n">
+        <v>0</v>
+      </c>
+      <c r="F320" t="n">
+        <v>2</v>
+      </c>
+      <c r="G320" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5892,6 +7816,12 @@
         <v>7</v>
       </c>
       <c r="E321" t="n">
+        <v>8</v>
+      </c>
+      <c r="F321" t="n">
+        <v>0</v>
+      </c>
+      <c r="G321" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5909,6 +7839,12 @@
         <v>9</v>
       </c>
       <c r="E322" t="n">
+        <v>6</v>
+      </c>
+      <c r="F322" t="n">
+        <v>0</v>
+      </c>
+      <c r="G322" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5926,6 +7862,12 @@
         <v>7</v>
       </c>
       <c r="E323" t="n">
+        <v>6</v>
+      </c>
+      <c r="F323" t="n">
+        <v>2</v>
+      </c>
+      <c r="G323" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5943,6 +7885,12 @@
         <v>9</v>
       </c>
       <c r="E324" t="n">
+        <v>6</v>
+      </c>
+      <c r="F324" t="n">
+        <v>1</v>
+      </c>
+      <c r="G324" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5960,6 +7908,12 @@
         <v>7</v>
       </c>
       <c r="E325" t="n">
+        <v>0</v>
+      </c>
+      <c r="F325" t="n">
+        <v>0</v>
+      </c>
+      <c r="G325" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5977,6 +7931,12 @@
         <v>7</v>
       </c>
       <c r="E326" t="n">
+        <v>1</v>
+      </c>
+      <c r="F326" t="n">
+        <v>0</v>
+      </c>
+      <c r="G326" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -5994,6 +7954,12 @@
         <v>7</v>
       </c>
       <c r="E327" t="n">
+        <v>2</v>
+      </c>
+      <c r="F327" t="n">
+        <v>1</v>
+      </c>
+      <c r="G327" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6011,6 +7977,12 @@
         <v>7</v>
       </c>
       <c r="E328" t="n">
+        <v>12</v>
+      </c>
+      <c r="F328" t="n">
+        <v>1</v>
+      </c>
+      <c r="G328" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6028,6 +8000,12 @@
         <v>9</v>
       </c>
       <c r="E329" t="n">
+        <v>9</v>
+      </c>
+      <c r="F329" t="n">
+        <v>0</v>
+      </c>
+      <c r="G329" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6045,6 +8023,12 @@
         <v>7</v>
       </c>
       <c r="E330" t="n">
+        <v>0</v>
+      </c>
+      <c r="F330" t="n">
+        <v>2</v>
+      </c>
+      <c r="G330" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6062,6 +8046,12 @@
         <v>7</v>
       </c>
       <c r="E331" t="n">
+        <v>9</v>
+      </c>
+      <c r="F331" t="n">
+        <v>3</v>
+      </c>
+      <c r="G331" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6079,6 +8069,12 @@
         <v>9</v>
       </c>
       <c r="E332" t="n">
+        <v>20</v>
+      </c>
+      <c r="F332" t="n">
+        <v>2</v>
+      </c>
+      <c r="G332" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6096,6 +8092,12 @@
         <v>7</v>
       </c>
       <c r="E333" t="n">
+        <v>3</v>
+      </c>
+      <c r="F333" t="n">
+        <v>3</v>
+      </c>
+      <c r="G333" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6113,6 +8115,12 @@
         <v>9</v>
       </c>
       <c r="E334" t="n">
+        <v>5</v>
+      </c>
+      <c r="F334" t="n">
+        <v>3</v>
+      </c>
+      <c r="G334" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6130,6 +8138,12 @@
         <v>7</v>
       </c>
       <c r="E335" t="n">
+        <v>1</v>
+      </c>
+      <c r="F335" t="n">
+        <v>0</v>
+      </c>
+      <c r="G335" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6147,6 +8161,12 @@
         <v>9</v>
       </c>
       <c r="E336" t="n">
+        <v>0</v>
+      </c>
+      <c r="F336" t="n">
+        <v>1</v>
+      </c>
+      <c r="G336" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6164,6 +8184,12 @@
         <v>7</v>
       </c>
       <c r="E337" t="n">
+        <v>9</v>
+      </c>
+      <c r="F337" t="n">
+        <v>0</v>
+      </c>
+      <c r="G337" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6181,6 +8207,12 @@
         <v>9</v>
       </c>
       <c r="E338" t="n">
+        <v>0</v>
+      </c>
+      <c r="F338" t="n">
+        <v>1</v>
+      </c>
+      <c r="G338" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6198,6 +8230,12 @@
         <v>7</v>
       </c>
       <c r="E339" t="n">
+        <v>7</v>
+      </c>
+      <c r="F339" t="n">
+        <v>0</v>
+      </c>
+      <c r="G339" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6215,6 +8253,12 @@
         <v>9</v>
       </c>
       <c r="E340" t="n">
+        <v>2</v>
+      </c>
+      <c r="F340" t="n">
+        <v>0</v>
+      </c>
+      <c r="G340" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6232,6 +8276,12 @@
         <v>7</v>
       </c>
       <c r="E341" t="n">
+        <v>3</v>
+      </c>
+      <c r="F341" t="n">
+        <v>0</v>
+      </c>
+      <c r="G341" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6249,6 +8299,12 @@
         <v>9</v>
       </c>
       <c r="E342" t="n">
+        <v>2</v>
+      </c>
+      <c r="F342" t="n">
+        <v>0</v>
+      </c>
+      <c r="G342" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6266,6 +8322,12 @@
         <v>7</v>
       </c>
       <c r="E343" t="n">
+        <v>5</v>
+      </c>
+      <c r="F343" t="n">
+        <v>1</v>
+      </c>
+      <c r="G343" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6283,6 +8345,12 @@
         <v>9</v>
       </c>
       <c r="E344" t="n">
+        <v>13</v>
+      </c>
+      <c r="F344" t="n">
+        <v>1</v>
+      </c>
+      <c r="G344" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6300,6 +8368,12 @@
         <v>7</v>
       </c>
       <c r="E345" t="n">
+        <v>1</v>
+      </c>
+      <c r="F345" t="n">
+        <v>1</v>
+      </c>
+      <c r="G345" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6317,6 +8391,12 @@
         <v>7</v>
       </c>
       <c r="E346" t="n">
+        <v>5</v>
+      </c>
+      <c r="F346" t="n">
+        <v>2</v>
+      </c>
+      <c r="G346" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6334,6 +8414,12 @@
         <v>9</v>
       </c>
       <c r="E347" t="n">
+        <v>5</v>
+      </c>
+      <c r="F347" t="n">
+        <v>2</v>
+      </c>
+      <c r="G347" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6351,6 +8437,12 @@
         <v>7</v>
       </c>
       <c r="E348" t="n">
+        <v>4</v>
+      </c>
+      <c r="F348" t="n">
+        <v>1</v>
+      </c>
+      <c r="G348" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6368,6 +8460,12 @@
         <v>9</v>
       </c>
       <c r="E349" t="n">
+        <v>2</v>
+      </c>
+      <c r="F349" t="n">
+        <v>0</v>
+      </c>
+      <c r="G349" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6385,6 +8483,12 @@
         <v>7</v>
       </c>
       <c r="E350" t="n">
+        <v>4</v>
+      </c>
+      <c r="F350" t="n">
+        <v>0</v>
+      </c>
+      <c r="G350" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6402,6 +8506,12 @@
         <v>9</v>
       </c>
       <c r="E351" t="n">
+        <v>3</v>
+      </c>
+      <c r="F351" t="n">
+        <v>1</v>
+      </c>
+      <c r="G351" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6419,6 +8529,12 @@
         <v>7</v>
       </c>
       <c r="E352" t="n">
+        <v>8</v>
+      </c>
+      <c r="F352" t="n">
+        <v>0</v>
+      </c>
+      <c r="G352" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6436,6 +8552,12 @@
         <v>9</v>
       </c>
       <c r="E353" t="n">
+        <v>4</v>
+      </c>
+      <c r="F353" t="n">
+        <v>0</v>
+      </c>
+      <c r="G353" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6453,6 +8575,12 @@
         <v>7</v>
       </c>
       <c r="E354" t="n">
+        <v>5</v>
+      </c>
+      <c r="F354" t="n">
+        <v>0</v>
+      </c>
+      <c r="G354" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6470,6 +8598,12 @@
         <v>7</v>
       </c>
       <c r="E355" t="n">
+        <v>4</v>
+      </c>
+      <c r="F355" t="n">
+        <v>1</v>
+      </c>
+      <c r="G355" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6487,6 +8621,12 @@
         <v>9</v>
       </c>
       <c r="E356" t="n">
+        <v>5</v>
+      </c>
+      <c r="F356" t="n">
+        <v>0</v>
+      </c>
+      <c r="G356" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6504,6 +8644,12 @@
         <v>7</v>
       </c>
       <c r="E357" t="n">
+        <v>1</v>
+      </c>
+      <c r="F357" t="n">
+        <v>0</v>
+      </c>
+      <c r="G357" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6521,6 +8667,12 @@
         <v>7</v>
       </c>
       <c r="E358" t="n">
+        <v>6</v>
+      </c>
+      <c r="F358" t="n">
+        <v>0</v>
+      </c>
+      <c r="G358" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6538,6 +8690,12 @@
         <v>9</v>
       </c>
       <c r="E359" t="n">
+        <v>3</v>
+      </c>
+      <c r="F359" t="n">
+        <v>1</v>
+      </c>
+      <c r="G359" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6555,6 +8713,12 @@
         <v>7</v>
       </c>
       <c r="E360" t="n">
+        <v>18</v>
+      </c>
+      <c r="F360" t="n">
+        <v>4</v>
+      </c>
+      <c r="G360" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6572,6 +8736,12 @@
         <v>9</v>
       </c>
       <c r="E361" t="n">
+        <v>12</v>
+      </c>
+      <c r="F361" t="n">
+        <v>1</v>
+      </c>
+      <c r="G361" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6589,6 +8759,12 @@
         <v>7</v>
       </c>
       <c r="E362" t="n">
+        <v>1</v>
+      </c>
+      <c r="F362" t="n">
+        <v>2</v>
+      </c>
+      <c r="G362" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6606,6 +8782,12 @@
         <v>9</v>
       </c>
       <c r="E363" t="n">
+        <v>6</v>
+      </c>
+      <c r="F363" t="n">
+        <v>1</v>
+      </c>
+      <c r="G363" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6623,6 +8805,12 @@
         <v>7</v>
       </c>
       <c r="E364" t="n">
+        <v>0</v>
+      </c>
+      <c r="F364" t="n">
+        <v>0</v>
+      </c>
+      <c r="G364" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6640,6 +8828,12 @@
         <v>7</v>
       </c>
       <c r="E365" t="n">
+        <v>11</v>
+      </c>
+      <c r="F365" t="n">
+        <v>0</v>
+      </c>
+      <c r="G365" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6657,6 +8851,12 @@
         <v>9</v>
       </c>
       <c r="E366" t="n">
+        <v>20</v>
+      </c>
+      <c r="F366" t="n">
+        <v>3</v>
+      </c>
+      <c r="G366" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6674,6 +8874,12 @@
         <v>7</v>
       </c>
       <c r="E367" t="n">
+        <v>4</v>
+      </c>
+      <c r="F367" t="n">
+        <v>0</v>
+      </c>
+      <c r="G367" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6691,6 +8897,12 @@
         <v>9</v>
       </c>
       <c r="E368" t="n">
+        <v>5</v>
+      </c>
+      <c r="F368" t="n">
+        <v>0</v>
+      </c>
+      <c r="G368" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6708,6 +8920,12 @@
         <v>7</v>
       </c>
       <c r="E369" t="n">
+        <v>1</v>
+      </c>
+      <c r="F369" t="n">
+        <v>2</v>
+      </c>
+      <c r="G369" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6725,6 +8943,12 @@
         <v>9</v>
       </c>
       <c r="E370" t="n">
+        <v>3</v>
+      </c>
+      <c r="F370" t="n">
+        <v>0</v>
+      </c>
+      <c r="G370" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6742,6 +8966,12 @@
         <v>7</v>
       </c>
       <c r="E371" t="n">
+        <v>7</v>
+      </c>
+      <c r="F371" t="n">
+        <v>3</v>
+      </c>
+      <c r="G371" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6759,6 +8989,12 @@
         <v>7</v>
       </c>
       <c r="E372" t="n">
+        <v>2</v>
+      </c>
+      <c r="F372" t="n">
+        <v>0</v>
+      </c>
+      <c r="G372" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6776,6 +9012,12 @@
         <v>7</v>
       </c>
       <c r="E373" t="n">
+        <v>5</v>
+      </c>
+      <c r="F373" t="n">
+        <v>4</v>
+      </c>
+      <c r="G373" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6793,6 +9035,12 @@
         <v>9</v>
       </c>
       <c r="E374" t="n">
+        <v>14</v>
+      </c>
+      <c r="F374" t="n">
+        <v>0</v>
+      </c>
+      <c r="G374" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6810,6 +9058,12 @@
         <v>7</v>
       </c>
       <c r="E375" t="n">
+        <v>11</v>
+      </c>
+      <c r="F375" t="n">
+        <v>1</v>
+      </c>
+      <c r="G375" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -6827,6 +9081,12 @@
         <v>9</v>
       </c>
       <c r="E376" t="n">
+        <v>12</v>
+      </c>
+      <c r="F376" t="n">
+        <v>1</v>
+      </c>
+      <c r="G376" t="n">
         <v>2000</v>
       </c>
     </row>

</xml_diff>